<commit_message>
Fix: Enterprise matrix was displayed last everywhere (dataset dict order)
The stored summary follows attack.json's dict order (ICS, Mobile,
Enterprise), so the largest and most relevant matrix appeared last in
the tiles, heatmap sections, list mini-bars, PDF scorecard/tactic
sections and XLSX rollups. Added a canonical display order
(enterprise, ics, mobile) — orderedDomains() in lib.ts and
_ordered_domains() in report.py — applied at every display site.
Computed numbers untouched.

Sample: the two disabled rules mapped to techniques other enabled rules
already covered, so Partial rendered as 0 and the state was
undemonstrable. Re-pointed them at T1070.004 and T1561.001 — the kit
now shows 2 partial.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample/MITRE_Sample/UploadSample/acme_sentinel_usecases.xlsx
+++ b/docs/sample/MITRE_Sample/UploadSample/acme_sentinel_usecases.xlsx
@@ -2318,7 +2318,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>T1485 - Data Destruction</t>
+          <t>T1561.001 - Disk Content Wipe</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -7498,7 +7498,7 @@
       </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
-          <t>T1562.001 - Disable or Modify Tools</t>
+          <t>T1070.004 - File Deletion</t>
         </is>
       </c>
       <c r="K109" s="2" t="inlineStr">

</xml_diff>